<commit_message>
v8: escalera reubicada, cocina abierta a la sala y puertas libres
- La escalera pasa a tener el pie en y=9,65 (huella 22 cm, meseta 88 cm, tramo de vuelta en losa con paso libre debajo): ya no tapa la cocina ni el baño grande.
- Cocina al centro (9,4 m²) abierta a la sala de estar por un paso libre de 1,60 m; dormitorio 2 al este; entradas de las dos plantas mayores; hueco superior en L.
- verificar_circulacion.py: comprueba sobre el GLB que se llega de cada estancia a las demás con 0,70 m (falla con v7, pasa con v8).
- Corregidos fallos de mobiliario que tapaban puertas (inodoro de la suite, armario del vestidor, sofá y armario de arriba, puertas sobre pilar y tabique).
- 16 paneles solares (uno tapaba el lucernario); DXF, instalaciones, mediciones, renders (dos interiores nuevos) y visor actualizados a v8.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GrFzVPJDRJqirwnmNdffa5
</commit_message>
<xml_diff>
--- a/cortijo/pedido_proveedores.xlsx
+++ b/cortijo/pedido_proveedores.xlsx
@@ -458,7 +458,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Ventanas, cristaleras y fijos (medidas del modelo v7, huecos de obra: ancho × alto en m)</t>
+          <t>Ventanas, cristaleras y fijos (medidas del modelo v8, huecos de obra: ancho × alto en m)</t>
         </is>
       </c>
     </row>
@@ -640,13 +640,13 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>1.2</v>
+        <v>1</v>
       </c>
       <c r="D7" t="n">
-        <v>1.3</v>
+        <v>1.1</v>
       </c>
       <c r="E7" t="n">
-        <v>0.9</v>
+        <v>1.1</v>
       </c>
       <c r="F7" t="n">
         <v>1</v>
@@ -830,13 +830,13 @@
         </is>
       </c>
       <c r="C12" t="n">
+        <v>1</v>
+      </c>
+      <c r="D12" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="E12" t="n">
         <v>0.9</v>
-      </c>
-      <c r="D12" t="n">
-        <v>1.1</v>
-      </c>
-      <c r="E12" t="n">
-        <v>1.1</v>
       </c>
       <c r="F12" t="n">
         <v>1</v>
@@ -1072,7 +1072,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>1</v>
+        <v>0.9</v>
       </c>
       <c r="D5" t="n">
         <v>2.1</v>
@@ -1258,7 +1258,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>0.8</v>
+        <v>0.75</v>
       </c>
       <c r="D11" t="n">
         <v>2.05</v>
@@ -1413,7 +1413,7 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>0.8</v>
+        <v>0.75</v>
       </c>
       <c r="D16" t="n">
         <v>2.05</v>
@@ -1994,16 +1994,16 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>1.6</v>
+        <v>1.4</v>
       </c>
       <c r="D20" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E20" t="n">
         <v>8.1</v>
       </c>
       <c r="F20" t="n">
-        <v>51.8</v>
+        <v>34</v>
       </c>
       <c r="G20" s="3" t="n"/>
       <c r="H20">
@@ -2023,16 +2023,16 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>1.4</v>
+        <v>1.3</v>
       </c>
       <c r="D21" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E21" t="n">
         <v>8.1</v>
       </c>
       <c r="F21" t="n">
-        <v>22.7</v>
+        <v>10.5</v>
       </c>
       <c r="G21" s="3" t="n"/>
       <c r="H21">
@@ -2052,16 +2052,16 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>1.3</v>
+        <v>1.6</v>
       </c>
       <c r="D22" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E22" t="n">
         <v>8.1</v>
       </c>
       <c r="F22" t="n">
-        <v>10.5</v>
+        <v>38.9</v>
       </c>
       <c r="G22" s="3" t="n"/>
       <c r="H22">
@@ -2114,17 +2114,17 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Barandilla de escalera y del hueco superior (≈ 9 m, estimado)</t>
+          <t>Barandillas: lado abierto de la escalera, suelo junto al hueco y pasamanos (≈ 10 m, estimado)</t>
         </is>
       </c>
       <c r="B25" t="inlineStr"/>
       <c r="C25" t="inlineStr"/>
       <c r="D25" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E25" t="inlineStr"/>
       <c r="F25" t="n">
-        <v>126</v>
+        <v>140</v>
       </c>
       <c r="G25" s="3" t="n"/>
       <c r="H25">
@@ -2135,17 +2135,17 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Soportes de 17 paneles solares, acero galvanizado (≈ 5 kg/panel, estimado)</t>
+          <t>Soportes de 16 paneles solares, acero galvanizado (≈ 5 kg/panel, estimado)</t>
         </is>
       </c>
       <c r="B26" t="inlineStr"/>
       <c r="C26" t="inlineStr"/>
       <c r="D26" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E26" t="inlineStr"/>
       <c r="F26" t="n">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="G26" s="3" t="n"/>
       <c r="H26">
@@ -2166,7 +2166,7 @@
       </c>
       <c r="E27" t="inlineStr"/>
       <c r="F27" t="n">
-        <v>109</v>
+        <v>108.9</v>
       </c>
       <c r="G27" s="3" t="n"/>
       <c r="H27">

</xml_diff>